<commit_message>
Refactor field and test data structures, expand product association in campaigns and orders, and standardize field names for interactions and orders. Updated tests accordingly to ensure consistency and maintainability.
</commit_message>
<xml_diff>
--- a/data/input/Low Level Field Detail Design(6).xlsx
+++ b/data/input/Low Level Field Detail Design(6).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://btgroupcloud.sharepoint.com/teams/CampaignManagementTransformation/Shared Documents/ROI and Attribution/Data Engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86C46C64-67AF-466A-917F-2A8852E2A9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB48945F-A91D-44AD-9ABB-43DC99024615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{EFC15C39-DC71-4D84-BB64-C304B1E6FB49}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="Interaction Types" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Attributes!$A$1:$J$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Attributes!$A$1:$J$164</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Channels!$A$1:$F$20</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -119,7 +119,7 @@
     See comment on product family</t>
       </text>
     </comment>
-    <comment ref="C93" authorId="6" shapeId="0" xr:uid="{B341755A-7D9C-4B12-B3E8-F721DABD8A3A}">
+    <comment ref="C91" authorId="6" shapeId="0" xr:uid="{B341755A-7D9C-4B12-B3E8-F721DABD8A3A}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1203" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="744">
   <si>
     <t>Name</t>
   </si>
@@ -973,7 +973,7 @@
     <t>???_owner</t>
   </si>
   <si>
-    <t>product_family</t>
+    <t>product_id</t>
   </si>
   <si>
     <t>Identifies the Product the Campaign Is Targeting</t>
@@ -1383,9 +1383,6 @@
     <t>* Should this differentiate the asset or be on the activity, Or actual a sub Object.</t>
   </si>
   <si>
-    <t>product_id</t>
-  </si>
-  <si>
     <t>Links to the product or product family that this asset is promoting.</t>
   </si>
   <si>
@@ -1425,28 +1422,19 @@
     <t>Unique Friendly name of the order, May be a concatenation of product, Time and company.</t>
   </si>
   <si>
-    <t>Which Product Family the product being sold in the order belongs to.</t>
+    <t>Which particular product was being sold in the order. *It might be actual we relate the order to a more complex product table depending on how the source data is structured</t>
+  </si>
+  <si>
+    <t>FK -&gt; Product.product_id</t>
+  </si>
+  <si>
+    <t>action_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In what part of the customer lifecycle is this order, what is its context based on current  company status. </t>
   </si>
   <si>
     <t>String Enum</t>
-  </si>
-  <si>
-    <t>product_group</t>
-  </si>
-  <si>
-    <t>Which product group the product being sold in the order belongs to.</t>
-  </si>
-  <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>Which particular product was being sold in the order. *It might be actual we relate the order to a more complex product table depending on how the source data is structured</t>
-  </si>
-  <si>
-    <t>action_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In what part of the customer lifecycle is this order, what is its context based on current  company status. </t>
   </si>
   <si>
     <t>"No Action", "Cease", "Modify", "Provide", "Mixed"</t>
@@ -1786,9 +1774,6 @@
   </si>
   <si>
     <t>Identifes the specific product that this change referers to.</t>
-  </si>
-  <si>
-    <t>Identifies the specific product family that this change refers to.</t>
   </si>
   <si>
     <t>sales_order_value_change</t>
@@ -6387,16 +6372,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D396AB2F-F9BE-4F78-8BC5-51EC98BD60B1}" name="Table1" displayName="Table1" ref="A1:J167" totalsRowShown="0">
-  <autoFilter ref="A1:J167" xr:uid="{AE1AD4F9-4E3A-41DA-9532-E435FAC78061}">
-    <filterColumn colId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D396AB2F-F9BE-4F78-8BC5-51EC98BD60B1}" name="Table1" displayName="Table1" ref="A1:J164" totalsRowShown="0">
+  <autoFilter ref="A1:J164" xr:uid="{AE1AD4F9-4E3A-41DA-9532-E435FAC78061}">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Orders"/>
+        <filter val="product"/>
+        <filter val="product_family"/>
+        <filter val="product_id"/>
+        <filter val="product_parent_id"/>
+        <filter val="product_price_type"/>
+        <filter val="product_quantity"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J165">
-    <sortCondition ref="A1:A165"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J162">
+    <sortCondition ref="A1:A162"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{FA10E4DE-EA14-4D6D-B2DE-B36300D4BF76}" name="Object" dataDxfId="2"/>
@@ -6788,7 +6778,7 @@
   <threadedComment ref="B61" dT="2025-03-07T22:24:32.38" personId="{B662DE40-7D09-46E5-994D-04657B702874}" id="{3477900C-1235-4AD9-B6B9-B36EBE216470}" parentId="{8497C7DA-1239-4373-88D7-CCD3FD1374B1}">
     <text>See comment on product family</text>
   </threadedComment>
-  <threadedComment ref="C93" dT="2025-03-06T16:36:49.39" personId="{14C944A1-1481-401E-974A-00A50AE6EDAF}" id="{B341755A-7D9C-4B12-B3E8-F721DABD8A3A}">
+  <threadedComment ref="C91" dT="2025-03-06T16:36:49.39" personId="{14C944A1-1481-401E-974A-00A50AE6EDAF}" id="{B341755A-7D9C-4B12-B3E8-F721DABD8A3A}">
     <text xml:space="preserve">@David Irvine 
 example please . is it a available field in existing Marketo Activities?
 </text>
@@ -7027,7 +7017,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="101.25">
+    <row r="7" spans="1:13" ht="105">
       <c r="A7" s="34" t="s">
         <v>42</v>
       </c>
@@ -7240,7 +7230,7 @@
       </c>
       <c r="G13">
         <f>COUNTIF(Attributes!A:A,objects!A13)</f>
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H13" t="s">
         <v>19</v>
@@ -7303,7 +7293,7 @@
       </c>
       <c r="G15">
         <f>COUNTIF(Attributes!A:A,objects!A15)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H15" t="s">
         <v>81</v>
@@ -7461,7 +7451,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1AD4F9-4E3A-41DA-9532-E435FAC78061}">
-  <dimension ref="A1:J167"/>
+  <dimension ref="A1:J164"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -7769,7 +7759,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="43.5" hidden="1">
+    <row r="20" spans="1:7" ht="45" hidden="1">
       <c r="A20" t="s">
         <v>155</v>
       </c>
@@ -7986,7 +7976,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="57.75" hidden="1">
+    <row r="34" spans="1:7" ht="60" hidden="1">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -8042,7 +8032,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -8056,7 +8046,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="130.5" hidden="1">
+    <row r="39" spans="1:7" ht="135" hidden="1">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -8115,7 +8105,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="43.5" hidden="1">
+    <row r="43" spans="1:7" ht="45" hidden="1">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -8135,7 +8125,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="72.75" hidden="1">
+    <row r="44" spans="1:7" ht="75" hidden="1">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -8152,7 +8142,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="43.5" hidden="1">
+    <row r="45" spans="1:7" ht="45" hidden="1">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -8202,7 +8192,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="24.75" hidden="1">
+    <row r="49" spans="1:10" ht="27" hidden="1">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -8364,27 +8354,27 @@
         <v>274</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="57.75" hidden="1">
+    <row r="61" spans="1:10" ht="60">
       <c r="A61" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B61" t="s">
+        <v>220</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="D61" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="D61" s="6" t="s">
+      <c r="E61" s="6" t="s">
         <v>277</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>278</v>
       </c>
       <c r="F61" t="s">
         <v>222</v>
       </c>
       <c r="J61" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="62" spans="1:10" hidden="1">
@@ -8392,10 +8382,10 @@
         <v>33</v>
       </c>
       <c r="B62" t="s">
+        <v>279</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>280</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>281</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -8405,10 +8395,10 @@
         <v>33</v>
       </c>
       <c r="B63" t="s">
+        <v>281</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -8418,26 +8408,26 @@
         <v>33</v>
       </c>
       <c r="B64" t="s">
+        <v>283</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>284</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>285</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" hidden="1">
       <c r="A65" t="s">
         <v>73</v>
       </c>
       <c r="B65" t="s">
+        <v>285</v>
+      </c>
+      <c r="C65" t="s">
         <v>286</v>
       </c>
-      <c r="C65" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10">
+    </row>
+    <row r="66" spans="1:10" hidden="1">
       <c r="A66" t="s">
         <v>73</v>
       </c>
@@ -8445,10 +8435,10 @@
         <v>231</v>
       </c>
       <c r="C66" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J66" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -8459,170 +8449,167 @@
         <v>220</v>
       </c>
       <c r="C67" t="s">
+        <v>288</v>
+      </c>
+      <c r="F67" t="s">
         <v>289</v>
       </c>
-      <c r="F67" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10">
+    </row>
+    <row r="68" spans="1:10" hidden="1">
       <c r="A68" t="s">
         <v>73</v>
       </c>
       <c r="B68" t="s">
+        <v>290</v>
+      </c>
+      <c r="C68" t="s">
         <v>291</v>
       </c>
-      <c r="C68" t="s">
+      <c r="F68" t="s">
         <v>292</v>
       </c>
-      <c r="F68" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10">
+      <c r="G68" s="16" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="45" hidden="1">
       <c r="A69" t="s">
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C69" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F69" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10">
+        <v>292</v>
+      </c>
+      <c r="G69" s="16" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" hidden="1">
       <c r="A70" t="s">
         <v>73</v>
       </c>
       <c r="B70" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C70" t="s">
-        <v>296</v>
-      </c>
-      <c r="F70" t="s">
-        <v>290</v>
-      </c>
-      <c r="G70" s="16" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="43.5">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" hidden="1">
       <c r="A71" t="s">
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C71" t="s">
-        <v>299</v>
-      </c>
-      <c r="F71" t="s">
-        <v>290</v>
-      </c>
-      <c r="G71" s="16" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" hidden="1">
       <c r="A72" t="s">
         <v>73</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="C72" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10">
+      <c r="C72"/>
+    </row>
+    <row r="73" spans="1:10" hidden="1">
       <c r="A73" t="s">
         <v>73</v>
       </c>
-      <c r="B73" t="s">
-        <v>303</v>
-      </c>
-      <c r="C73" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10">
+      <c r="B73" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C73"/>
+    </row>
+    <row r="74" spans="1:10" hidden="1">
       <c r="A74" t="s">
         <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C74"/>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" hidden="1">
       <c r="A75" t="s">
         <v>73</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C75"/>
     </row>
-    <row r="76" spans="1:10">
-      <c r="A76" t="s">
+    <row r="76" spans="1:10" hidden="1">
+      <c r="A76" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C76"/>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" hidden="1">
       <c r="A77" t="s">
         <v>73</v>
       </c>
-      <c r="B77" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="C77"/>
-    </row>
-    <row r="78" spans="1:10">
+      <c r="B77" t="s">
+        <v>133</v>
+      </c>
+      <c r="C77" t="s">
+        <v>306</v>
+      </c>
+      <c r="F77" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" hidden="1">
       <c r="A78" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="C78"/>
-    </row>
-    <row r="79" spans="1:10">
+        <v>307</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="F78" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" hidden="1">
       <c r="A79" t="s">
         <v>73</v>
       </c>
       <c r="B79" t="s">
-        <v>133</v>
+        <v>309</v>
       </c>
       <c r="C79" t="s">
         <v>310</v>
       </c>
-      <c r="F79" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10">
-      <c r="A80" s="4" t="s">
+    </row>
+    <row r="80" spans="1:10" hidden="1">
+      <c r="A80" t="s">
         <v>73</v>
       </c>
-      <c r="B80" s="4" t="s">
+      <c r="B80" t="s">
         <v>311</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>312</v>
       </c>
       <c r="F80" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" hidden="1">
       <c r="A81" t="s">
         <v>73</v>
       </c>
@@ -8632,60 +8619,60 @@
       <c r="C81" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="82" spans="1:10">
+      <c r="F81" t="s">
+        <v>315</v>
+      </c>
+      <c r="J81" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" hidden="1">
       <c r="A82" t="s">
         <v>73</v>
       </c>
       <c r="B82" t="s">
-        <v>315</v>
-      </c>
-      <c r="C82" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="F82" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10">
+      <c r="C82" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" hidden="1">
       <c r="A83" t="s">
         <v>73</v>
       </c>
       <c r="B83" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C83" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F83" t="s">
-        <v>319</v>
-      </c>
-      <c r="J83" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10">
-      <c r="A84" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" hidden="1">
+      <c r="A84" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B84" t="s">
-        <v>320</v>
-      </c>
-      <c r="C84" t="s">
+      <c r="B84" s="4" t="s">
         <v>321</v>
       </c>
+      <c r="C84" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="J84" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="85" spans="1:10">
-      <c r="A85" t="s">
+      <c r="A85" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B85" t="s">
-        <v>322</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="B85" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="F85" t="s">
+      <c r="C85" s="4" t="s">
         <v>324</v>
       </c>
     </row>
@@ -8696,67 +8683,76 @@
       <c r="B86" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="C86" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="J86" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10">
+      <c r="C86" s="4"/>
+    </row>
+    <row r="87" spans="1:10" hidden="1">
       <c r="A87" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B87" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C87" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="C87" s="4" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10">
+    </row>
+    <row r="88" spans="1:10" hidden="1">
       <c r="A88" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B88" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="C88" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="C88" s="4"/>
-    </row>
-    <row r="89" spans="1:10">
-      <c r="A89" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B89" s="4" t="s">
+    </row>
+    <row r="89" spans="1:10" hidden="1">
+      <c r="A89" t="s">
+        <v>42</v>
+      </c>
+      <c r="B89" t="s">
         <v>330</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="90" spans="1:10">
-      <c r="A90" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B90" s="4" t="s">
+      <c r="D89" t="s">
         <v>332</v>
       </c>
-      <c r="C90" s="4" t="s">
+    </row>
+    <row r="90" spans="1:10" hidden="1">
+      <c r="A90" t="s">
+        <v>42</v>
+      </c>
+      <c r="B90" t="s">
+        <v>179</v>
+      </c>
+      <c r="C90" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="91" spans="1:10" hidden="1">
+      <c r="F90" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="45" hidden="1">
       <c r="A91" t="s">
         <v>42</v>
       </c>
       <c r="B91" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C91" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D91" t="s">
-        <v>336</v>
+        <v>337</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="F91" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="92" spans="1:10" hidden="1">
@@ -8764,33 +8760,21 @@
         <v>42</v>
       </c>
       <c r="B92" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C92" t="s">
-        <v>337</v>
-      </c>
-      <c r="F92" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" ht="29.25" hidden="1">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" hidden="1">
       <c r="A93" t="s">
         <v>42</v>
       </c>
       <c r="B93" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C93" t="s">
-        <v>340</v>
-      </c>
-      <c r="D93" t="s">
-        <v>341</v>
-      </c>
-      <c r="E93" s="6" t="s">
         <v>342</v>
-      </c>
-      <c r="F93" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="94" spans="1:10" hidden="1">
@@ -8798,10 +8782,10 @@
         <v>42</v>
       </c>
       <c r="B94" t="s">
-        <v>187</v>
-      </c>
-      <c r="C94" t="s">
-        <v>344</v>
+        <v>265</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="95" spans="1:10" hidden="1">
@@ -8809,10 +8793,10 @@
         <v>42</v>
       </c>
       <c r="B95" t="s">
-        <v>345</v>
+        <v>231</v>
       </c>
       <c r="C95" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="96" spans="1:10" hidden="1">
@@ -8820,10 +8804,16 @@
         <v>42</v>
       </c>
       <c r="B96" t="s">
-        <v>265</v>
-      </c>
-      <c r="C96" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C96" t="s">
+        <v>346</v>
+      </c>
+      <c r="D96" t="s">
         <v>347</v>
+      </c>
+      <c r="E96" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="97" spans="1:6" hidden="1">
@@ -8831,9 +8821,15 @@
         <v>42</v>
       </c>
       <c r="B97" t="s">
-        <v>231</v>
+        <v>349</v>
       </c>
       <c r="C97" t="s">
+        <v>350</v>
+      </c>
+      <c r="D97" t="s">
+        <v>347</v>
+      </c>
+      <c r="E97" t="s">
         <v>348</v>
       </c>
     </row>
@@ -8842,16 +8838,10 @@
         <v>42</v>
       </c>
       <c r="B98" t="s">
-        <v>349</v>
-      </c>
-      <c r="C98" t="s">
-        <v>350</v>
-      </c>
-      <c r="D98" t="s">
-        <v>351</v>
-      </c>
-      <c r="E98" t="s">
-        <v>352</v>
+        <v>283</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="99" spans="1:6" hidden="1">
@@ -8859,16 +8849,10 @@
         <v>42</v>
       </c>
       <c r="B99" t="s">
-        <v>353</v>
-      </c>
-      <c r="C99" t="s">
-        <v>354</v>
-      </c>
-      <c r="D99" t="s">
-        <v>351</v>
-      </c>
-      <c r="E99" t="s">
-        <v>352</v>
+        <v>281</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="100" spans="1:6" hidden="1">
@@ -8876,10 +8860,10 @@
         <v>42</v>
       </c>
       <c r="B100" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="101" spans="1:6" hidden="1">
@@ -8887,10 +8871,10 @@
         <v>42</v>
       </c>
       <c r="B101" t="s">
-        <v>282</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>283</v>
+        <v>185</v>
+      </c>
+      <c r="C101" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="102" spans="1:6" hidden="1">
@@ -8898,10 +8882,10 @@
         <v>42</v>
       </c>
       <c r="B102" t="s">
-        <v>280</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>281</v>
+        <v>352</v>
+      </c>
+      <c r="C102" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="103" spans="1:6" hidden="1">
@@ -8909,10 +8893,13 @@
         <v>42</v>
       </c>
       <c r="B103" t="s">
-        <v>185</v>
+        <v>354</v>
       </c>
       <c r="C103" t="s">
         <v>355</v>
+      </c>
+      <c r="D103" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="104" spans="1:6" hidden="1">
@@ -8925,6 +8912,9 @@
       <c r="C104" t="s">
         <v>357</v>
       </c>
+      <c r="F104" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="105" spans="1:6" hidden="1">
       <c r="A105" t="s">
@@ -8936,36 +8926,36 @@
       <c r="C105" t="s">
         <v>359</v>
       </c>
-      <c r="D105" t="s">
-        <v>207</v>
+      <c r="F105" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="106" spans="1:6" hidden="1">
       <c r="A106" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="B106" t="s">
+        <v>231</v>
+      </c>
+      <c r="C106" t="s">
         <v>360</v>
       </c>
-      <c r="C106" t="s">
-        <v>361</v>
-      </c>
       <c r="F106" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="107" spans="1:6" hidden="1">
       <c r="A107" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="B107" t="s">
+        <v>361</v>
+      </c>
+      <c r="C107" t="s">
         <v>362</v>
       </c>
-      <c r="C107" t="s">
-        <v>363</v>
-      </c>
       <c r="F107" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
     </row>
     <row r="108" spans="1:6" hidden="1">
@@ -8973,52 +8963,47 @@
         <v>28</v>
       </c>
       <c r="B108" t="s">
-        <v>231</v>
+        <v>363</v>
       </c>
       <c r="C108" t="s">
         <v>364</v>
       </c>
       <c r="F108" t="s">
-        <v>159</v>
+        <v>365</v>
       </c>
     </row>
     <row r="109" spans="1:6" hidden="1">
       <c r="A109" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B109" t="s">
-        <v>365</v>
+        <v>136</v>
       </c>
       <c r="C109" t="s">
         <v>366</v>
       </c>
-      <c r="F109" t="s">
-        <v>159</v>
-      </c>
     </row>
     <row r="110" spans="1:6" hidden="1">
       <c r="A110" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B110" t="s">
         <v>367</v>
       </c>
-      <c r="C110" t="s">
-        <v>368</v>
-      </c>
-      <c r="F110" t="s">
-        <v>369</v>
-      </c>
+      <c r="C110"/>
     </row>
     <row r="111" spans="1:6" hidden="1">
       <c r="A111" t="s">
         <v>58</v>
       </c>
       <c r="B111" t="s">
-        <v>136</v>
-      </c>
-      <c r="C111" t="s">
-        <v>370</v>
+        <v>279</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="F111" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="112" spans="1:6" hidden="1">
@@ -9026,58 +9011,59 @@
         <v>58</v>
       </c>
       <c r="B112" t="s">
-        <v>371</v>
-      </c>
-      <c r="C112"/>
+        <v>281</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="F112" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="113" spans="1:10" hidden="1">
       <c r="A113" t="s">
         <v>58</v>
       </c>
       <c r="B113" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F113" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="114" spans="1:10" hidden="1">
-      <c r="A114" t="s">
-        <v>58</v>
-      </c>
       <c r="B114" t="s">
-        <v>282</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="F114" t="s">
-        <v>159</v>
+        <v>370</v>
+      </c>
+      <c r="C114" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="115" spans="1:10" hidden="1">
       <c r="A115" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B115" t="s">
-        <v>284</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>285</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="C115"/>
       <c r="F115" t="s">
-        <v>373</v>
+        <v>138</v>
       </c>
     </row>
     <row r="116" spans="1:10" hidden="1">
+      <c r="A116" t="s">
+        <v>68</v>
+      </c>
       <c r="B116" t="s">
-        <v>374</v>
-      </c>
-      <c r="C116" t="s">
-        <v>375</v>
+        <v>133</v>
+      </c>
+      <c r="C116"/>
+      <c r="F116" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="117" spans="1:10" hidden="1">
@@ -9085,11 +9071,16 @@
         <v>68</v>
       </c>
       <c r="B117" t="s">
-        <v>136</v>
-      </c>
-      <c r="C117"/>
+        <v>185</v>
+      </c>
+      <c r="C117" t="s">
+        <v>372</v>
+      </c>
       <c r="F117" t="s">
-        <v>138</v>
+        <v>163</v>
+      </c>
+      <c r="J117" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="118" spans="1:10" hidden="1">
@@ -9097,11 +9088,16 @@
         <v>68</v>
       </c>
       <c r="B118" t="s">
-        <v>133</v>
-      </c>
-      <c r="C118"/>
+        <v>187</v>
+      </c>
+      <c r="C118" t="s">
+        <v>373</v>
+      </c>
       <c r="F118" t="s">
-        <v>135</v>
+        <v>163</v>
+      </c>
+      <c r="J118" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="119" spans="1:10" hidden="1">
@@ -9109,47 +9105,37 @@
         <v>68</v>
       </c>
       <c r="B119" t="s">
-        <v>185</v>
+        <v>375</v>
       </c>
       <c r="C119" t="s">
         <v>376</v>
       </c>
       <c r="F119" t="s">
-        <v>163</v>
-      </c>
-      <c r="J119" t="s">
-        <v>279</v>
+        <v>129</v>
       </c>
     </row>
     <row r="120" spans="1:10" hidden="1">
       <c r="A120" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B120" t="s">
-        <v>187</v>
-      </c>
-      <c r="C120" t="s">
-        <v>377</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="C120"/>
       <c r="F120" t="s">
-        <v>163</v>
-      </c>
-      <c r="J120" t="s">
-        <v>378</v>
+        <v>120</v>
       </c>
     </row>
     <row r="121" spans="1:10" hidden="1">
       <c r="A121" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B121" t="s">
-        <v>379</v>
-      </c>
-      <c r="C121" t="s">
-        <v>380</v>
-      </c>
+        <v>377</v>
+      </c>
+      <c r="C121"/>
       <c r="F121" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="122" spans="1:10" hidden="1">
@@ -9157,23 +9143,22 @@
         <v>63</v>
       </c>
       <c r="B122" t="s">
-        <v>133</v>
+        <v>378</v>
       </c>
       <c r="C122"/>
-      <c r="F122" t="s">
-        <v>120</v>
-      </c>
     </row>
     <row r="123" spans="1:10" hidden="1">
       <c r="A123" t="s">
         <v>63</v>
       </c>
       <c r="B123" t="s">
+        <v>379</v>
+      </c>
+      <c r="C123" t="s">
+        <v>380</v>
+      </c>
+      <c r="G123" s="16" t="s">
         <v>381</v>
-      </c>
-      <c r="C123"/>
-      <c r="F123" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="124" spans="1:10" hidden="1">
@@ -9183,68 +9168,65 @@
       <c r="B124" t="s">
         <v>382</v>
       </c>
-      <c r="C124"/>
+      <c r="C124" t="s">
+        <v>383</v>
+      </c>
     </row>
     <row r="125" spans="1:10" hidden="1">
       <c r="A125" t="s">
         <v>63</v>
       </c>
-      <c r="B125" t="s">
-        <v>383</v>
-      </c>
-      <c r="C125" t="s">
+      <c r="B125" s="4" t="s">
         <v>384</v>
       </c>
-      <c r="G125" s="16" t="s">
-        <v>385</v>
-      </c>
+      <c r="C125"/>
     </row>
     <row r="126" spans="1:10" hidden="1">
       <c r="A126" t="s">
         <v>63</v>
       </c>
       <c r="B126" t="s">
-        <v>386</v>
-      </c>
-      <c r="C126" t="s">
-        <v>387</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="C126"/>
     </row>
     <row r="127" spans="1:10" hidden="1">
       <c r="A127" t="s">
         <v>63</v>
       </c>
-      <c r="B127" s="4" t="s">
+      <c r="B127" t="s">
+        <v>386</v>
+      </c>
+      <c r="C127" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" hidden="1">
+      <c r="B128" t="s">
+        <v>370</v>
+      </c>
+      <c r="C128" t="s">
         <v>388</v>
       </c>
-      <c r="C127"/>
-    </row>
-    <row r="128" spans="1:10" hidden="1">
-      <c r="A128" t="s">
-        <v>63</v>
-      </c>
-      <c r="B128" t="s">
-        <v>389</v>
-      </c>
-      <c r="C128"/>
     </row>
     <row r="129" spans="1:7" hidden="1">
       <c r="A129" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="B129" t="s">
-        <v>390</v>
-      </c>
-      <c r="C129" t="s">
-        <v>391</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="C129"/>
     </row>
     <row r="130" spans="1:7" hidden="1">
+      <c r="A130" t="s">
+        <v>37</v>
+      </c>
       <c r="B130" t="s">
-        <v>374</v>
+        <v>231</v>
       </c>
       <c r="C130" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="131" spans="1:7" hidden="1">
@@ -9252,19 +9234,21 @@
         <v>37</v>
       </c>
       <c r="B131" t="s">
-        <v>334</v>
-      </c>
-      <c r="C131"/>
+        <v>241</v>
+      </c>
+      <c r="C131" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="132" spans="1:7" hidden="1">
       <c r="A132" t="s">
         <v>37</v>
       </c>
       <c r="B132" t="s">
-        <v>231</v>
+        <v>391</v>
       </c>
       <c r="C132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="133" spans="1:7" hidden="1">
@@ -9272,83 +9256,86 @@
         <v>37</v>
       </c>
       <c r="B133" t="s">
-        <v>241</v>
+        <v>393</v>
       </c>
       <c r="C133" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="134" spans="1:7" hidden="1">
-      <c r="A134" t="s">
+    <row r="134" spans="1:7" s="4" customFormat="1" hidden="1">
+      <c r="A134" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C134" s="4" t="s">
         <v>396</v>
       </c>
+      <c r="D134" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="E134" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="G134" s="6"/>
     </row>
     <row r="135" spans="1:7" hidden="1">
       <c r="A135" t="s">
         <v>37</v>
       </c>
       <c r="B135" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C135" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" s="4" customFormat="1" hidden="1">
-      <c r="A136" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" hidden="1">
+      <c r="A136" t="s">
         <v>37</v>
       </c>
-      <c r="B136" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="C136" s="4" t="s">
+      <c r="B136" t="s">
         <v>400</v>
       </c>
-      <c r="D136" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="E136" s="4" t="s">
+      <c r="C136" t="s">
         <v>401</v>
       </c>
-      <c r="G136" s="6"/>
     </row>
     <row r="137" spans="1:7" hidden="1">
-      <c r="A137" t="s">
-        <v>37</v>
-      </c>
-      <c r="B137" t="s">
+      <c r="A137" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="C137" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="C137" t="s">
+    </row>
+    <row r="138" spans="1:7" hidden="1">
+      <c r="A138" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="C138" s="5" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1">
-      <c r="A138" t="s">
-        <v>37</v>
-      </c>
-      <c r="B138" t="s">
-        <v>404</v>
-      </c>
-      <c r="C138" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" hidden="1">
+    <row r="139" spans="1:7">
       <c r="A139" s="4" t="s">
         <v>82</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>345</v>
+        <v>220</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
+      </c>
+      <c r="F139" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="140" spans="1:7" hidden="1">
@@ -9356,10 +9343,10 @@
         <v>82</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>246</v>
+        <v>405</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="141" spans="1:7" hidden="1">
@@ -9367,7 +9354,7 @@
         <v>82</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>293</v>
+        <v>407</v>
       </c>
       <c r="C141" s="5" t="s">
         <v>408</v>
@@ -9378,10 +9365,10 @@
         <v>82</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>220</v>
+        <v>409</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="143" spans="1:7" hidden="1">
@@ -9389,21 +9376,24 @@
         <v>82</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" hidden="1">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="60" hidden="1">
       <c r="A144" s="4" t="s">
         <v>82</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>413</v>
+        <v>414</v>
+      </c>
+      <c r="G144" s="16" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="145" spans="1:7" hidden="1">
@@ -9411,10 +9401,10 @@
         <v>82</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="146" spans="1:7" hidden="1">
@@ -9422,57 +9412,72 @@
         <v>82</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" ht="57.75" hidden="1">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" hidden="1">
       <c r="A147" s="4" t="s">
         <v>82</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>418</v>
+        <v>133</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="G147" s="16" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="148" spans="1:7" hidden="1">
-      <c r="A148" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B148" s="4" t="s">
+    <row r="148" spans="1:7">
+      <c r="A148" t="s">
+        <v>100</v>
+      </c>
+      <c r="B148" t="s">
+        <v>220</v>
+      </c>
+      <c r="C148" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="C148" s="5" t="s">
+      <c r="D148" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="149" spans="1:7" hidden="1">
-      <c r="A149" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B149" s="4" t="s">
+      <c r="E148" t="s">
         <v>423</v>
       </c>
-      <c r="C149" s="5" t="s">
+      <c r="F148" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7">
+      <c r="A149" t="s">
+        <v>100</v>
+      </c>
+      <c r="B149" t="s">
         <v>424</v>
       </c>
+      <c r="C149" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="D149" t="s">
+        <v>426</v>
+      </c>
+      <c r="F149" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="150" spans="1:7" hidden="1">
-      <c r="A150" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B150" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C150" s="5" t="s">
-        <v>425</v>
+      <c r="A150" t="s">
+        <v>100</v>
+      </c>
+      <c r="B150" t="s">
+        <v>231</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="F150" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="151" spans="1:7" hidden="1">
@@ -9480,19 +9485,16 @@
         <v>100</v>
       </c>
       <c r="B151" t="s">
-        <v>275</v>
+        <v>429</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="D151" t="s">
-        <v>427</v>
-      </c>
-      <c r="E151" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F151" t="s">
-        <v>120</v>
+        <v>129</v>
+      </c>
+      <c r="G151" s="16" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="152" spans="1:7" hidden="1">
@@ -9500,16 +9502,13 @@
         <v>100</v>
       </c>
       <c r="B152" t="s">
-        <v>429</v>
+        <v>279</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="D152" t="s">
-        <v>431</v>
+        <v>280</v>
       </c>
       <c r="F152" t="s">
-        <v>432</v>
+        <v>368</v>
       </c>
     </row>
     <row r="153" spans="1:7" hidden="1">
@@ -9517,10 +9516,10 @@
         <v>100</v>
       </c>
       <c r="B153" t="s">
-        <v>231</v>
+        <v>281</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>433</v>
+        <v>282</v>
       </c>
       <c r="F153" t="s">
         <v>159</v>
@@ -9531,58 +9530,46 @@
         <v>100</v>
       </c>
       <c r="B154" t="s">
-        <v>434</v>
+        <v>283</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>435</v>
+        <v>284</v>
       </c>
       <c r="F154" t="s">
-        <v>129</v>
-      </c>
-      <c r="G154" s="16" t="s">
-        <v>436</v>
+        <v>369</v>
       </c>
     </row>
     <row r="155" spans="1:7" hidden="1">
       <c r="A155" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B155" t="s">
-        <v>280</v>
+        <v>432</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="F155" t="s">
-        <v>372</v>
+        <v>433</v>
       </c>
     </row>
     <row r="156" spans="1:7" hidden="1">
       <c r="A156" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B156" t="s">
-        <v>282</v>
+        <v>246</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="F156" t="s">
-        <v>159</v>
+        <v>434</v>
       </c>
     </row>
     <row r="157" spans="1:7" hidden="1">
       <c r="A157" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B157" t="s">
-        <v>284</v>
+        <v>435</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="F157" t="s">
-        <v>373</v>
+        <v>436</v>
       </c>
     </row>
     <row r="158" spans="1:7" hidden="1">
@@ -9601,10 +9588,10 @@
         <v>105</v>
       </c>
       <c r="B159" t="s">
-        <v>246</v>
+        <v>439</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="160" spans="1:7" hidden="1">
@@ -9612,9 +9599,6 @@
         <v>105</v>
       </c>
       <c r="B160" t="s">
-        <v>440</v>
-      </c>
-      <c r="C160" s="1" t="s">
         <v>441</v>
       </c>
     </row>
@@ -9625,79 +9609,49 @@
       <c r="B161" t="s">
         <v>442</v>
       </c>
-      <c r="C161" s="1" t="s">
-        <v>443</v>
-      </c>
     </row>
     <row r="162" spans="1:7" hidden="1">
       <c r="A162" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="B162" t="s">
+        <v>443</v>
+      </c>
+      <c r="C162" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="C162" s="1" t="s">
+      <c r="F162" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" hidden="1">
+      <c r="A163" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B163" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="30" hidden="1">
+      <c r="A164" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B164" t="s">
         <v>445</v>
       </c>
-    </row>
-    <row r="163" spans="1:7" hidden="1">
-      <c r="A163" t="s">
-        <v>105</v>
-      </c>
-      <c r="B163" t="s">
+      <c r="C164" s="1" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="164" spans="1:7" hidden="1">
-      <c r="A164" t="s">
-        <v>105</v>
-      </c>
-      <c r="B164" t="s">
+      <c r="E164" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="165" spans="1:7" hidden="1">
-      <c r="A165" t="s">
-        <v>28</v>
-      </c>
-      <c r="B165" t="s">
+      <c r="G164" s="16" t="s">
         <v>448</v>
       </c>
-      <c r="C165" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="F165" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7" hidden="1">
-      <c r="A166" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B166" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" ht="29.25" hidden="1">
-      <c r="A167" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B167" t="s">
-        <v>450</v>
-      </c>
-      <c r="C167" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="E167" t="s">
-        <v>452</v>
-      </c>
-      <c r="G167" s="16" t="s">
-        <v>453</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J107">
-    <sortCondition ref="A2:A107"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J105">
+    <sortCondition ref="A2:A105"/>
   </sortState>
   <dataValidations count="1">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1" xr:uid="{EAF3A632-FFC2-461F-8E3C-46D4F5CA1EA8}"/>
@@ -9741,55 +9695,55 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>453</v>
+      </c>
+      <c r="F1" s="31" t="s">
         <v>454</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="E1" s="31" t="s">
-        <v>458</v>
-      </c>
-      <c r="F1" s="31" t="s">
-        <v>459</v>
       </c>
       <c r="G1" t="s">
         <v>63</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="K1" t="s">
+        <v>457</v>
+      </c>
+      <c r="M1" t="s">
+        <v>458</v>
+      </c>
+      <c r="N1" t="s">
+        <v>459</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="K1" t="s">
+      <c r="R1" s="4" t="s">
         <v>462</v>
       </c>
-      <c r="M1" t="s">
+      <c r="S1" s="4" t="s">
         <v>463</v>
       </c>
-      <c r="N1" t="s">
+      <c r="T1" s="4" t="s">
         <v>464</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>465</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -9800,10 +9754,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="E2" s="31">
         <v>1</v>
@@ -9815,7 +9769,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="I2" s="3">
         <v>10</v>
@@ -9839,10 +9793,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="E3" s="31">
         <v>1</v>
@@ -9854,7 +9808,7 @@
         <v>2</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="I3" s="3">
         <v>200</v>
@@ -9878,10 +9832,10 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="E4" s="31">
         <v>2</v>
@@ -9891,7 +9845,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="I4" s="3">
         <v>15</v>
@@ -9915,10 +9869,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="E5" s="31">
         <v>3</v>
@@ -9928,7 +9882,7 @@
         <v>4</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="I5" s="3">
         <v>1</v>
@@ -9955,7 +9909,7 @@
         <v>73</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="E6" s="31">
         <v>4</v>
@@ -9967,7 +9921,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="I6" s="3">
         <v>0</v>
@@ -9994,7 +9948,7 @@
         <v>73</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="E7" s="31"/>
       <c r="F7" s="31">
@@ -10004,7 +9958,7 @@
         <v>6</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="I7" s="3">
         <v>256</v>
@@ -10031,7 +9985,7 @@
         <v>73</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="E8" s="31">
         <v>6</v>
@@ -10041,7 +9995,7 @@
         <v>7</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="I8" s="3">
         <v>24</v>
@@ -10068,7 +10022,7 @@
         <v>73</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="E9" s="31"/>
       <c r="F9" s="31">
@@ -10078,7 +10032,7 @@
         <v>8</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="I9" s="3">
         <v>51</v>
@@ -10117,78 +10071,78 @@
         <v>0</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="10" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" s="17" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="11" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="11" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="D4" s="17"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="11" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="11" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="11" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="D7" s="17"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="10" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -10196,47 +10150,47 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="11" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="D9" s="17"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="11" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="D10" s="17"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="11" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="D11" s="17"/>
     </row>
     <row r="12" spans="1:4" ht="30">
       <c r="A12" s="11" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="D12" s="17"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="10" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -10244,724 +10198,724 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="11" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="D14" s="17"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="11" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="D15" s="17"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="11" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="D16" s="17"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="11" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="D17" s="17"/>
     </row>
     <row r="18" spans="1:6">
       <c r="E18" s="13" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="45">
       <c r="A19" s="12" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="30">
       <c r="A20" s="12" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="60">
       <c r="A21" s="12" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="30">
       <c r="A22" s="12" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="135">
       <c r="A23" s="12" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
       <c r="B23" s="16" t="s">
+        <v>529</v>
+      </c>
+      <c r="C23" s="16" t="s">
         <v>534</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>539</v>
-      </c>
       <c r="E23" s="14" t="s">
-        <v>540</v>
+        <v>535</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>541</v>
+        <v>536</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="270">
       <c r="A24" s="12" t="s">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>543</v>
+        <v>538</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>544</v>
+        <v>539</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>545</v>
+        <v>540</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="75">
       <c r="A25" s="12" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>548</v>
+        <v>543</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>550</v>
+        <v>545</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="120">
       <c r="A26" s="12" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="B26" s="16" t="s">
+        <v>542</v>
+      </c>
+      <c r="C26" s="16" t="s">
         <v>547</v>
       </c>
-      <c r="C26" s="16" t="s">
-        <v>552</v>
-      </c>
       <c r="E26" s="14" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="75">
       <c r="A27" s="12" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>556</v>
+        <v>551</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="75">
       <c r="A28" s="12" t="s">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="75">
       <c r="A29" s="12" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="75">
       <c r="A30" s="12" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="75">
       <c r="A31" s="12" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="45">
       <c r="A32" s="12" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="C32" s="19"/>
       <c r="E32" s="14" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>574</v>
+        <v>569</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="30">
       <c r="A33" s="12" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="30">
       <c r="A34" s="12" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>582</v>
+        <v>577</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="12" t="s">
-        <v>583</v>
+        <v>578</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>584</v>
+        <v>579</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="12" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>590</v>
+        <v>585</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="12" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="B37" s="16" t="s">
+        <v>583</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>587</v>
+      </c>
+      <c r="E37" s="14" t="s">
         <v>588</v>
       </c>
-      <c r="C37" s="16" t="s">
-        <v>592</v>
-      </c>
-      <c r="E37" s="14" t="s">
-        <v>593</v>
-      </c>
       <c r="F37" s="8" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="12" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>598</v>
+        <v>593</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="12" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>600</v>
+        <v>595</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>601</v>
+        <v>596</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="45">
       <c r="A40" s="12" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="60">
       <c r="A41" s="12" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="60">
       <c r="A42" s="12" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="45">
       <c r="A43" s="12" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="30">
       <c r="A44" s="12" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="105">
       <c r="A45" s="12" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="45">
       <c r="A46" s="12" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="B46" s="21" t="s">
+        <v>621</v>
+      </c>
+      <c r="E46" s="14" t="s">
         <v>626</v>
       </c>
-      <c r="E46" s="14" t="s">
-        <v>631</v>
-      </c>
       <c r="F46" s="8" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="30">
       <c r="A47" s="12" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="30">
       <c r="A48" s="12" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="B48" s="23" t="s">
+        <v>629</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>633</v>
+      </c>
+      <c r="F48" s="15" t="s">
         <v>634</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>638</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="12" t="s">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="B49" s="21" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="B50" s="21" t="s">
+        <v>636</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>640</v>
+      </c>
+      <c r="F50" s="8" t="s">
         <v>641</v>
-      </c>
-      <c r="E50" s="14" t="s">
-        <v>645</v>
-      </c>
-      <c r="F50" s="8" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="60">
       <c r="A51" s="12" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="60">
       <c r="A52" s="12" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="B52" s="23" t="s">
+        <v>643</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>647</v>
+      </c>
+      <c r="F52" s="8" t="s">
         <v>648</v>
-      </c>
-      <c r="E52" s="14" t="s">
-        <v>652</v>
-      </c>
-      <c r="F52" s="8" t="s">
-        <v>653</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="12" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="B53" s="22" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="165">
       <c r="A54" s="12" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="30">
       <c r="A55" s="12" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="B55" s="23" t="s">
+        <v>654</v>
+      </c>
+      <c r="C55" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="C55" s="16" t="s">
-        <v>664</v>
-      </c>
       <c r="E55" s="14" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="60">
       <c r="A57" s="12" t="s">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="B57" s="23" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="60">
       <c r="A58" s="12" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="B58" s="23" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="45">
       <c r="A59" s="12" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B59" s="21" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="E59" s="14" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="45">
       <c r="A60" s="12" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="B60" s="23" t="s">
-        <v>680</v>
+        <v>675</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>681</v>
+        <v>676</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>682</v>
+        <v>677</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="45">
       <c r="A61" s="12" t="s">
-        <v>683</v>
+        <v>678</v>
       </c>
       <c r="B61" s="23" t="s">
+        <v>675</v>
+      </c>
+      <c r="E61" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="F61" s="8" t="s">
         <v>680</v>
-      </c>
-      <c r="E61" s="14" t="s">
-        <v>684</v>
-      </c>
-      <c r="F61" s="8" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="45">
       <c r="A62" s="12" t="s">
-        <v>686</v>
+        <v>681</v>
       </c>
       <c r="B62" s="23" t="s">
-        <v>680</v>
+        <v>675</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
     </row>
   </sheetData>
@@ -10982,234 +10936,234 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="D1" t="s">
-        <v>691</v>
+        <v>686</v>
       </c>
       <c r="E1" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="F1" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="C2" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D2" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="C3" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D3" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="C4" t="s">
+        <v>690</v>
+      </c>
+      <c r="D4" t="s">
         <v>695</v>
-      </c>
-      <c r="D4" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="C5" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D5" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
       <c r="F5" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="B6" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="C6" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D6" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="B7" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="C7" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D7" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="B8" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="C8" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D8" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="C9" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D9" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="C10" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D10" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="B11" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="C11" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D11" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="B12" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="C12" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D12" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="B13" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
       <c r="C13" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D13" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="B14" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="C14" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D14" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="B15" t="s">
-        <v>715</v>
+        <v>710</v>
       </c>
       <c r="C15" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D15" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="B16" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="C16" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D16" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="17" spans="2:8">
       <c r="B17" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="C17" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="D17" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="18" spans="2:8">
       <c r="B18" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="C18" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="D18" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="19" spans="2:8">
       <c r="B19" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="C19" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="D19" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="20" spans="2:8">
       <c r="B20" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="C20" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="D20" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="22" spans="2:8">
@@ -11242,7 +11196,7 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="28" t="s">
-        <v>722</v>
+        <v>717</v>
       </c>
       <c r="B1" s="39" t="s">
         <v>47</v>
@@ -11256,353 +11210,353 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="29" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="B2" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="C2" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="D2" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="29" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="B3" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="C3" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="D3" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="H3" s="25"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="29" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="B4" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
       <c r="C4" t="s">
-        <v>727</v>
+        <v>722</v>
       </c>
       <c r="D4" t="s">
+        <v>720</v>
+      </c>
+      <c r="E4" t="s">
+        <v>723</v>
+      </c>
+      <c r="F4" t="s">
+        <v>724</v>
+      </c>
+      <c r="G4" t="s">
         <v>725</v>
-      </c>
-      <c r="E4" t="s">
-        <v>728</v>
-      </c>
-      <c r="F4" t="s">
-        <v>729</v>
-      </c>
-      <c r="G4" t="s">
-        <v>730</v>
       </c>
       <c r="H4" s="25"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="29" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="B5" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="H5" s="25"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="29" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="B6" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="C6" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="D6" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="H6" s="25"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="29" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="B7" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="C7" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="D7" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="E7" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H7" s="25"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="29" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="B8" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C8" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="D8" t="s">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="H8" s="25"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="29" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="B9" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C9" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="H9" s="25"/>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="29" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="B10" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C10" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="D10" t="s">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="H10" s="25"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="29" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="B11" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C11" t="s">
-        <v>737</v>
+        <v>732</v>
       </c>
       <c r="D11" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="H11" s="25"/>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="29" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="B12" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C12" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="D12" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="E12" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="F12" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="G12" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H12" s="25"/>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="29" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
       <c r="B13" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C13" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="D13" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="E13" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="F13" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="G13" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H13" s="25"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="29" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="B14" t="s">
+        <v>731</v>
+      </c>
+      <c r="C14" t="s">
+        <v>734</v>
+      </c>
+      <c r="D14" t="s">
+        <v>733</v>
+      </c>
+      <c r="E14" t="s">
         <v>736</v>
       </c>
-      <c r="C14" t="s">
-        <v>739</v>
-      </c>
-      <c r="D14" t="s">
-        <v>738</v>
-      </c>
-      <c r="E14" t="s">
-        <v>741</v>
-      </c>
       <c r="F14" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="G14" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="29" t="s">
-        <v>715</v>
+        <v>710</v>
       </c>
       <c r="B15" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C15" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="D15" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="E15" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="F15" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="G15" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H15" s="25"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="29" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="B16" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C16" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="D16" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="E16" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="F16" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="G16" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="29" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="B17" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C17" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="E17" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="H17" s="25"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="29" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="B18" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="C18" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="H18" s="25"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="29" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="B19" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="C19" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="D19" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="H19" s="25"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="29" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="B20" t="s">
+        <v>731</v>
+      </c>
+      <c r="C20" t="s">
+        <v>734</v>
+      </c>
+      <c r="D20" t="s">
+        <v>733</v>
+      </c>
+      <c r="E20" t="s">
         <v>736</v>
       </c>
-      <c r="C20" t="s">
-        <v>739</v>
-      </c>
-      <c r="D20" t="s">
-        <v>738</v>
-      </c>
-      <c r="E20" t="s">
-        <v>741</v>
-      </c>
       <c r="F20" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="G20" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="H20" s="25" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="30" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="C21" s="26"/>
       <c r="D21" s="26"/>
@@ -11620,6 +11574,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D1F78A46A5B61544A3F5E5F9D558353B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd5889db134979e54dcf054cdc4727ec">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7019f60-298e-442e-b6f6-687001478962" xmlns:ns3="244a3a2d-c3b8-4eaa-9334-4c3b8cbc7cc9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdf5543a8e45e11fa247a01810ff6e7b" ns2:_="" ns3:_="">
     <xsd:import namespace="a7019f60-298e-442e-b6f6-687001478962"/>
@@ -11820,7 +11780,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -11829,20 +11789,14 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{981D98BA-C602-41F7-9CF6-ADC2B2B0572D}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221E8208-2559-4473-AFD3-FB4000FD0DD1}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51BB428E-D1CA-47E8-B784-F33B49A13D8D}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{981D98BA-C602-41F7-9CF6-ADC2B2B0572D}"/>
 </file>
</xml_diff>

<commit_message>
Refactor person-company role generator to handle filtered row counts during role assignment and enhance start/end date logic. Add a new script to analyze attribution linking table, and update dependencies in `poetry.lock` to include additional data processing libraries.
</commit_message>
<xml_diff>
--- a/data/input/Low Level Field Detail Design(6).xlsx
+++ b/data/input/Low Level Field Detail Design(6).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://btgroupcloud.sharepoint.com/teams/CampaignManagementTransformation/Shared Documents/ROI and Attribution/Data Engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA6B9540-07E2-4BC7-BE4A-5E7C961D53C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9CABA46-BF39-46C6-A7D5-944861D4720A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{EFC15C39-DC71-4D84-BB64-C304B1E6FB49}"/>
   </bookViews>
@@ -7077,6 +7077,7 @@
     <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="28" customWidth="1"/>
     <col min="12" max="12" width="31.85546875" customWidth="1"/>
     <col min="13" max="13" width="22.28515625" customWidth="1"/>
@@ -7321,7 +7322,7 @@
         <v>15</v>
       </c>
       <c r="J7">
-        <v>10000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="72.599999999999994">
@@ -7354,7 +7355,7 @@
         <v>17</v>
       </c>
       <c r="J8">
-        <v>500000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="29.1">
@@ -7420,7 +7421,7 @@
         <v>7</v>
       </c>
       <c r="J10">
-        <v>5000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="87">
@@ -7453,7 +7454,7 @@
         <v>6</v>
       </c>
       <c r="J11">
-        <v>3000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="57.95">
@@ -7519,7 +7520,7 @@
         <v>9</v>
       </c>
       <c r="J13">
-        <v>7000</v>
+        <v>7000000</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="101.45">
@@ -12419,21 +12420,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D1F78A46A5B61544A3F5E5F9D558353B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd5889db134979e54dcf054cdc4727ec">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7019f60-298e-442e-b6f6-687001478962" xmlns:ns3="244a3a2d-c3b8-4eaa-9334-4c3b8cbc7cc9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdf5543a8e45e11fa247a01810ff6e7b" ns2:_="" ns3:_="">
     <xsd:import namespace="a7019f60-298e-442e-b6f6-687001478962"/>
@@ -12634,8 +12620,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51BB428E-D1CA-47E8-B784-F33B49A13D8D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221E8208-2559-4473-AFD3-FB4000FD0DD1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12643,5 +12644,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221E8208-2559-4473-AFD3-FB4000FD0DD1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51BB428E-D1CA-47E8-B784-F33B49A13D8D}"/>
 </file>
</xml_diff>

<commit_message>
Add lazy pipelines with streaming joins for improved memory efficiency, enhance attribution linking with detailed timings, expand link generation methods, and update dependencies in `poetry.lock`.
Signed-off-by: David Irvine <Dirvine@clever-touch.com>
</commit_message>
<xml_diff>
--- a/data/input/Low Level Field Detail Design(6).xlsx
+++ b/data/input/Low Level Field Detail Design(6).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://btgroupcloud.sharepoint.com/teams/CampaignManagementTransformation/Shared Documents/ROI and Attribution/Data Engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9CABA46-BF39-46C6-A7D5-944861D4720A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F159CB11-530D-4788-8D07-F07A13A7A3ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{EFC15C39-DC71-4D84-BB64-C304B1E6FB49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" xr2:uid="{EFC15C39-DC71-4D84-BB64-C304B1E6FB49}"/>
   </bookViews>
   <sheets>
     <sheet name="objects" sheetId="1" r:id="rId1"/>
@@ -6631,8 +6631,7 @@
   <autoFilter ref="A1:J167" xr:uid="{AE1AD4F9-4E3A-41DA-9532-E435FAC78061}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Attribution Model Output Table"/>
-        <filter val="Attrribution Model"/>
+        <filter val="Orders"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -7066,7 +7065,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF98BEB6-65EB-437D-B437-4DFA85EC4A08}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.42578125" bestFit="1" customWidth="1"/>
@@ -7124,7 +7123,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="72.599999999999994">
+    <row r="2" spans="1:13" ht="90">
       <c r="A2" s="31" t="s">
         <v>13</v>
       </c>
@@ -7160,7 +7159,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="72.599999999999994">
+    <row r="3" spans="1:13" ht="75">
       <c r="A3" s="32" t="s">
         <v>21</v>
       </c>
@@ -7193,7 +7192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="72.599999999999994">
+    <row r="4" spans="1:13" ht="75">
       <c r="A4" s="32" t="s">
         <v>28</v>
       </c>
@@ -7226,7 +7225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="57.95">
+    <row r="5" spans="1:13" ht="60">
       <c r="A5" s="9" t="s">
         <v>33</v>
       </c>
@@ -7259,7 +7258,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="43.5">
+    <row r="6" spans="1:13" ht="60">
       <c r="A6" s="7" t="s">
         <v>37</v>
       </c>
@@ -7292,7 +7291,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="101.45">
+    <row r="7" spans="1:13" ht="105">
       <c r="A7" s="31" t="s">
         <v>42</v>
       </c>
@@ -7325,7 +7324,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="72.599999999999994">
+    <row r="8" spans="1:13" ht="105">
       <c r="A8" s="31" t="s">
         <v>47</v>
       </c>
@@ -7358,7 +7357,7 @@
         <v>5000000</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="29.1">
+    <row r="9" spans="1:13" ht="30">
       <c r="A9" s="7" t="s">
         <v>52</v>
       </c>
@@ -7391,7 +7390,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="57.95">
+    <row r="10" spans="1:13" ht="75">
       <c r="A10" s="31" t="s">
         <v>59</v>
       </c>
@@ -7424,7 +7423,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="87">
+    <row r="11" spans="1:13" ht="120">
       <c r="A11" s="31" t="s">
         <v>64</v>
       </c>
@@ -7457,7 +7456,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="57.95">
+    <row r="12" spans="1:13" ht="60">
       <c r="A12" s="34" t="s">
         <v>69</v>
       </c>
@@ -7490,7 +7489,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="43.5">
+    <row r="13" spans="1:13" ht="45">
       <c r="A13" s="31" t="s">
         <v>74</v>
       </c>
@@ -7520,10 +7519,10 @@
         <v>9</v>
       </c>
       <c r="J13">
-        <v>7000000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="101.45">
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="105">
       <c r="A14" s="31" t="s">
         <v>79</v>
       </c>
@@ -7553,7 +7552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="57.95">
+    <row r="15" spans="1:13" ht="60">
       <c r="A15" s="7" t="s">
         <v>83</v>
       </c>
@@ -7583,7 +7582,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="43.5">
+    <row r="16" spans="1:13" ht="45">
       <c r="A16" s="7" t="s">
         <v>87</v>
       </c>
@@ -7613,7 +7612,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="57.95">
+    <row r="17" spans="1:10" ht="60">
       <c r="A17" s="3" t="s">
         <v>90</v>
       </c>
@@ -7646,7 +7645,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="57.95">
+    <row r="18" spans="1:10" ht="75">
       <c r="A18" s="3" t="s">
         <v>96</v>
       </c>
@@ -7705,7 +7704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="43.5">
+    <row r="20" spans="1:10" ht="45">
       <c r="A20" s="3" t="s">
         <v>106</v>
       </c>
@@ -7739,8 +7738,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1AD4F9-4E3A-41DA-9532-E435FAC78061}">
-  <dimension ref="A1:J171"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:J167"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.85546875" bestFit="1" customWidth="1"/>
@@ -7915,7 +7914,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" hidden="1">
       <c r="A11" t="s">
         <v>90</v>
       </c>
@@ -7929,7 +7928,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" hidden="1">
       <c r="A12" t="s">
         <v>90</v>
       </c>
@@ -7943,7 +7942,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" hidden="1">
       <c r="A13" t="s">
         <v>90</v>
       </c>
@@ -7957,7 +7956,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" hidden="1">
       <c r="A14" t="s">
         <v>90</v>
       </c>
@@ -7974,7 +7973,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" hidden="1">
       <c r="A15" t="s">
         <v>156</v>
       </c>
@@ -7988,7 +7987,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" hidden="1">
       <c r="A16" t="s">
         <v>156</v>
       </c>
@@ -8005,7 +8004,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" hidden="1">
       <c r="A17" t="s">
         <v>156</v>
       </c>
@@ -8019,7 +8018,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" hidden="1">
       <c r="A18" t="s">
         <v>156</v>
       </c>
@@ -8033,7 +8032,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" hidden="1">
       <c r="A19" t="s">
         <v>156</v>
       </c>
@@ -8047,7 +8046,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="43.5">
+    <row r="20" spans="1:7" ht="45" hidden="1">
       <c r="A20" t="s">
         <v>156</v>
       </c>
@@ -8070,7 +8069,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" hidden="1">
       <c r="A21" t="s">
         <v>156</v>
       </c>
@@ -8087,7 +8086,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" hidden="1">
       <c r="A22" t="s">
         <v>156</v>
       </c>
@@ -8264,7 +8263,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="57.95" hidden="1">
+    <row r="34" spans="1:7" ht="60" hidden="1">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -8334,7 +8333,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="130.5" hidden="1">
+    <row r="39" spans="1:7" ht="135" hidden="1">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -8393,7 +8392,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="43.5" hidden="1">
+    <row r="43" spans="1:7" ht="45" hidden="1">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -8413,7 +8412,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="72.599999999999994" hidden="1">
+    <row r="44" spans="1:7" ht="75" hidden="1">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -8430,7 +8429,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="43.5" hidden="1">
+    <row r="45" spans="1:7" ht="45" hidden="1">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -8480,7 +8479,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="26.45" hidden="1">
+    <row r="49" spans="1:10" ht="27" hidden="1">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -8642,7 +8641,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="57.95" hidden="1">
+    <row r="61" spans="1:10" ht="60" hidden="1">
       <c r="A61" s="4" t="s">
         <v>33</v>
       </c>
@@ -8704,7 +8703,7 @@
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
     </row>
-    <row r="65" spans="1:10" hidden="1">
+    <row r="65" spans="1:10">
       <c r="A65" t="s">
         <v>74</v>
       </c>
@@ -8715,7 +8714,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1">
+    <row r="66" spans="1:10">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -8729,7 +8728,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1">
+    <row r="67" spans="1:10">
       <c r="A67" t="s">
         <v>74</v>
       </c>
@@ -8743,7 +8742,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="68" spans="1:10" hidden="1">
+    <row r="68" spans="1:10">
       <c r="A68" t="s">
         <v>74</v>
       </c>
@@ -8760,7 +8759,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="43.5" hidden="1">
+    <row r="69" spans="1:10" ht="45">
       <c r="A69" t="s">
         <v>74</v>
       </c>
@@ -8777,7 +8776,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1">
+    <row r="70" spans="1:10">
       <c r="A70" t="s">
         <v>74</v>
       </c>
@@ -8788,7 +8787,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1">
+    <row r="71" spans="1:10">
       <c r="A71" t="s">
         <v>74</v>
       </c>
@@ -8799,7 +8798,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1">
+    <row r="72" spans="1:10">
       <c r="A72" t="s">
         <v>74</v>
       </c>
@@ -8808,7 +8807,7 @@
       </c>
       <c r="C72"/>
     </row>
-    <row r="73" spans="1:10" hidden="1">
+    <row r="73" spans="1:10">
       <c r="A73" t="s">
         <v>74</v>
       </c>
@@ -8817,7 +8816,7 @@
       </c>
       <c r="C73"/>
     </row>
-    <row r="74" spans="1:10" hidden="1">
+    <row r="74" spans="1:10">
       <c r="A74" t="s">
         <v>74</v>
       </c>
@@ -8826,7 +8825,7 @@
       </c>
       <c r="C74"/>
     </row>
-    <row r="75" spans="1:10" hidden="1">
+    <row r="75" spans="1:10">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -8835,7 +8834,7 @@
       </c>
       <c r="C75"/>
     </row>
-    <row r="76" spans="1:10" hidden="1">
+    <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
         <v>74</v>
       </c>
@@ -8844,7 +8843,7 @@
       </c>
       <c r="C76"/>
     </row>
-    <row r="77" spans="1:10" hidden="1">
+    <row r="77" spans="1:10">
       <c r="A77" t="s">
         <v>74</v>
       </c>
@@ -8858,7 +8857,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1">
+    <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
         <v>74</v>
       </c>
@@ -8872,7 +8871,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1">
+    <row r="79" spans="1:10">
       <c r="A79" t="s">
         <v>74</v>
       </c>
@@ -8883,7 +8882,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1">
+    <row r="80" spans="1:10">
       <c r="A80" t="s">
         <v>74</v>
       </c>
@@ -8897,7 +8896,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1">
+    <row r="81" spans="1:10">
       <c r="A81" t="s">
         <v>74</v>
       </c>
@@ -8914,7 +8913,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="82" spans="1:10" hidden="1">
+    <row r="82" spans="1:10">
       <c r="A82" t="s">
         <v>74</v>
       </c>
@@ -8925,7 +8924,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="83" spans="1:10" hidden="1">
+    <row r="83" spans="1:10">
       <c r="A83" t="s">
         <v>74</v>
       </c>
@@ -8939,7 +8938,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="84" spans="1:10" hidden="1">
+    <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
         <v>74</v>
       </c>
@@ -8953,7 +8952,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="85" spans="1:10" hidden="1">
+    <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
         <v>74</v>
       </c>
@@ -8964,7 +8963,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="86" spans="1:10" hidden="1">
+    <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
         <v>74</v>
       </c>
@@ -8973,7 +8972,7 @@
       </c>
       <c r="C86" s="4"/>
     </row>
-    <row r="87" spans="1:10" hidden="1">
+    <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
         <v>74</v>
       </c>
@@ -8984,7 +8983,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1">
+    <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
         <v>74</v>
       </c>
@@ -9023,7 +9022,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="15" hidden="1">
+    <row r="91" spans="1:10" hidden="1">
       <c r="A91" s="3" t="s">
         <v>42</v>
       </c>
@@ -9031,7 +9030,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="29.25" hidden="1">
+    <row r="92" spans="1:10" ht="45" hidden="1">
       <c r="A92" t="s">
         <v>42</v>
       </c>
@@ -9051,7 +9050,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="15" hidden="1">
+    <row r="93" spans="1:10" hidden="1">
       <c r="A93" t="s">
         <v>42</v>
       </c>
@@ -9062,7 +9061,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="15" hidden="1">
+    <row r="94" spans="1:10" hidden="1">
       <c r="A94" t="s">
         <v>42</v>
       </c>
@@ -9073,7 +9072,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="15" hidden="1">
+    <row r="95" spans="1:10" hidden="1">
       <c r="A95" t="s">
         <v>42</v>
       </c>
@@ -9084,7 +9083,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="15" hidden="1">
+    <row r="96" spans="1:10" hidden="1">
       <c r="A96" t="s">
         <v>42</v>
       </c>
@@ -9095,7 +9094,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="15" hidden="1">
+    <row r="97" spans="1:6" hidden="1">
       <c r="A97" t="s">
         <v>42</v>
       </c>
@@ -9112,7 +9111,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="15" hidden="1">
+    <row r="98" spans="1:6" hidden="1">
       <c r="A98" t="s">
         <v>42</v>
       </c>
@@ -9129,7 +9128,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="15" hidden="1">
+    <row r="99" spans="1:6" hidden="1">
       <c r="A99" t="s">
         <v>42</v>
       </c>
@@ -9140,7 +9139,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="15" hidden="1">
+    <row r="100" spans="1:6" hidden="1">
       <c r="A100" t="s">
         <v>42</v>
       </c>
@@ -9151,7 +9150,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="15" hidden="1">
+    <row r="101" spans="1:6" hidden="1">
       <c r="A101" t="s">
         <v>42</v>
       </c>
@@ -9162,7 +9161,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="15" hidden="1">
+    <row r="102" spans="1:6" hidden="1">
       <c r="A102" t="s">
         <v>42</v>
       </c>
@@ -9173,7 +9172,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="15" hidden="1">
+    <row r="103" spans="1:6" hidden="1">
       <c r="A103" t="s">
         <v>42</v>
       </c>
@@ -9184,7 +9183,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="15" hidden="1">
+    <row r="104" spans="1:6" hidden="1">
       <c r="A104" t="s">
         <v>42</v>
       </c>
@@ -9198,7 +9197,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="15" hidden="1">
+    <row r="105" spans="1:6" hidden="1">
       <c r="A105" t="s">
         <v>42</v>
       </c>
@@ -9494,7 +9493,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="29.1" hidden="1">
+    <row r="126" spans="1:10" ht="30" hidden="1">
       <c r="A126" t="s">
         <v>64</v>
       </c>
@@ -9646,7 +9645,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="29.1" hidden="1">
+    <row r="138" spans="1:7" ht="30" hidden="1">
       <c r="A138" s="4" t="s">
         <v>83</v>
       </c>
@@ -9715,7 +9714,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="57.95" hidden="1">
+    <row r="144" spans="1:7" ht="60" hidden="1">
       <c r="A144" s="4" t="s">
         <v>83</v>
       </c>
@@ -9729,7 +9728,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="29.1" hidden="1">
+    <row r="145" spans="1:7" ht="30" hidden="1">
       <c r="A145" s="4" t="s">
         <v>83</v>
       </c>
@@ -9740,7 +9739,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="29.1" hidden="1">
+    <row r="146" spans="1:7" ht="30" hidden="1">
       <c r="A146" s="4" t="s">
         <v>83</v>
       </c>
@@ -9957,7 +9956,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="15" hidden="1">
+    <row r="163" spans="1:7" hidden="1">
       <c r="A163" t="s">
         <v>42</v>
       </c>
@@ -9971,7 +9970,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="29.1" hidden="1">
+    <row r="164" spans="1:7" ht="30" hidden="1">
       <c r="A164" s="3" t="s">
         <v>21</v>
       </c>
@@ -10008,7 +10007,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="29.25" hidden="1">
+    <row r="166" spans="1:7" ht="30" hidden="1">
       <c r="A166" s="39" t="s">
         <v>52</v>
       </c>
@@ -10028,7 +10027,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="29.25" hidden="1">
+    <row r="167" spans="1:7" ht="30" hidden="1">
       <c r="A167" s="39" t="s">
         <v>52</v>
       </c>
@@ -10048,8 +10047,6 @@
         <v>474</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="15"/>
-    <row r="171" spans="1:7" ht="15"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J105">
     <sortCondition ref="A2:A105"/>
@@ -10081,7 +10078,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FEA969B-2E99-43A3-91BB-BD5F9824B477}">
   <dimension ref="A1:T9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" customWidth="1"/>
@@ -10457,7 +10454,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2AC8CA7-C3B2-4113-BDC9-28FC11714663}">
   <dimension ref="A1:F62"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="47.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" style="16" customWidth="1"/>
@@ -10467,7 +10464,7 @@
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" ht="30">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10579,7 +10576,7 @@
       </c>
       <c r="D11" s="17"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" ht="30">
       <c r="A12" s="11" t="s">
         <v>526</v>
       </c>
@@ -10645,7 +10642,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="43.5">
+    <row r="19" spans="1:6" ht="45">
       <c r="A19" s="12" t="s">
         <v>539</v>
       </c>
@@ -10662,7 +10659,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="29.1">
+    <row r="20" spans="1:6" ht="30">
       <c r="A20" s="12" t="s">
         <v>544</v>
       </c>
@@ -10679,7 +10676,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="57.95">
+    <row r="21" spans="1:6" ht="60">
       <c r="A21" s="12" t="s">
         <v>507</v>
       </c>
@@ -10699,7 +10696,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29.1">
+    <row r="22" spans="1:6" ht="30">
       <c r="A22" s="12" t="s">
         <v>554</v>
       </c>
@@ -10716,7 +10713,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="130.5">
+    <row r="23" spans="1:6" ht="135">
       <c r="A23" s="12" t="s">
         <v>559</v>
       </c>
@@ -10733,7 +10730,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="231.95">
+    <row r="24" spans="1:6" ht="270">
       <c r="A24" s="12" t="s">
         <v>563</v>
       </c>
@@ -10750,7 +10747,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="57.95">
+    <row r="25" spans="1:6" ht="75">
       <c r="A25" s="12" t="s">
         <v>567</v>
       </c>
@@ -10767,7 +10764,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="116.1">
+    <row r="26" spans="1:6" ht="120">
       <c r="A26" s="12" t="s">
         <v>572</v>
       </c>
@@ -10784,7 +10781,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="57.95">
+    <row r="27" spans="1:6" ht="75">
       <c r="A27" s="12" t="s">
         <v>576</v>
       </c>
@@ -10798,7 +10795,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="57.95">
+    <row r="28" spans="1:6" ht="75">
       <c r="A28" s="12" t="s">
         <v>579</v>
       </c>
@@ -10812,7 +10809,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="57.95">
+    <row r="29" spans="1:6" ht="75">
       <c r="A29" s="12" t="s">
         <v>582</v>
       </c>
@@ -10826,7 +10823,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="57.95">
+    <row r="30" spans="1:6" ht="75">
       <c r="A30" s="12" t="s">
         <v>585</v>
       </c>
@@ -10840,7 +10837,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="57.95">
+    <row r="31" spans="1:6" ht="75">
       <c r="A31" s="12" t="s">
         <v>588</v>
       </c>
@@ -10857,7 +10854,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="43.5">
+    <row r="32" spans="1:6" ht="45">
       <c r="A32" s="12" t="s">
         <v>592</v>
       </c>
@@ -10872,7 +10869,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" ht="30">
       <c r="A33" s="12" t="s">
         <v>596</v>
       </c>
@@ -10886,7 +10883,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="29.1">
+    <row r="34" spans="1:6" ht="30">
       <c r="A34" s="12" t="s">
         <v>600</v>
       </c>
@@ -10979,7 +10976,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="29.1">
+    <row r="40" spans="1:6" ht="45">
       <c r="A40" s="12" t="s">
         <v>623</v>
       </c>
@@ -10993,7 +10990,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="57.95">
+    <row r="41" spans="1:6" ht="60">
       <c r="A41" s="12" t="s">
         <v>627</v>
       </c>
@@ -11007,7 +11004,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="43.5">
+    <row r="42" spans="1:6" ht="60">
       <c r="A42" s="12" t="s">
         <v>631</v>
       </c>
@@ -11024,7 +11021,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="43.5">
+    <row r="43" spans="1:6" ht="45">
       <c r="A43" s="12" t="s">
         <v>636</v>
       </c>
@@ -11041,7 +11038,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="29.1">
+    <row r="44" spans="1:6" ht="30">
       <c r="A44" s="12" t="s">
         <v>641</v>
       </c>
@@ -11058,7 +11055,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="101.45">
+    <row r="45" spans="1:6" ht="105">
       <c r="A45" s="12" t="s">
         <v>646</v>
       </c>
@@ -11075,7 +11072,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="29.1">
+    <row r="46" spans="1:6" ht="45">
       <c r="A46" s="12" t="s">
         <v>651</v>
       </c>
@@ -11089,7 +11086,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" ht="30">
       <c r="A47" s="12" t="s">
         <v>654</v>
       </c>
@@ -11103,7 +11100,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" ht="30">
       <c r="A48" s="12" t="s">
         <v>658</v>
       </c>
@@ -11145,7 +11142,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="43.5">
+    <row r="51" spans="1:6" ht="60">
       <c r="A51" s="12" t="s">
         <v>668</v>
       </c>
@@ -11159,7 +11156,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="43.5">
+    <row r="52" spans="1:6" ht="60">
       <c r="A52" s="12" t="s">
         <v>672</v>
       </c>
@@ -11187,7 +11184,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="130.5">
+    <row r="54" spans="1:6" ht="165">
       <c r="A54" s="12" t="s">
         <v>679</v>
       </c>
@@ -11204,7 +11201,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="29.1">
+    <row r="55" spans="1:6" ht="30">
       <c r="A55" s="12" t="s">
         <v>684</v>
       </c>
@@ -11235,7 +11232,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="43.5">
+    <row r="57" spans="1:6" ht="60">
       <c r="A57" s="12" t="s">
         <v>691</v>
       </c>
@@ -11249,7 +11246,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="43.5">
+    <row r="58" spans="1:6" ht="60">
       <c r="A58" s="12" t="s">
         <v>694</v>
       </c>
@@ -11263,7 +11260,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="29.1">
+    <row r="59" spans="1:6" ht="45">
       <c r="A59" s="12" t="s">
         <v>697</v>
       </c>
@@ -11277,7 +11274,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="43.5">
+    <row r="60" spans="1:6" ht="45">
       <c r="A60" s="12" t="s">
         <v>700</v>
       </c>
@@ -11291,7 +11288,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="43.5">
+    <row r="61" spans="1:6" ht="45">
       <c r="A61" s="12" t="s">
         <v>704</v>
       </c>
@@ -11305,7 +11302,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="43.5">
+    <row r="62" spans="1:6" ht="45">
       <c r="A62" s="12" t="s">
         <v>707</v>
       </c>
@@ -11328,7 +11325,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8D126A-E50F-4373-9159-5B9100CAC9A2}">
   <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="32.28515625" customWidth="1"/>
     <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
@@ -11677,7 +11674,7 @@
         <v>Sent;Received;Clicked</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="15">
+    <row r="18" spans="2:8">
       <c r="B18" t="s">
         <v>746</v>
       </c>
@@ -11695,7 +11692,7 @@
         <v>Attempted;Answered;Conversed</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15">
+    <row r="19" spans="2:8">
       <c r="B19" t="s">
         <v>748</v>
       </c>
@@ -11804,7 +11801,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EAF728D-8DC4-43CB-A2BE-8E22F440F4CC}">
   <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="61.85546875" bestFit="1" customWidth="1"/>
@@ -11816,7 +11813,7 @@
     <col min="10" max="10" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15">
+    <row r="1" spans="1:10">
       <c r="A1" s="40" t="s">
         <v>755</v>
       </c>
@@ -11848,7 +11845,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15">
+    <row r="2" spans="1:10">
       <c r="A2" s="44" t="s">
         <v>716</v>
       </c>
@@ -11871,7 +11868,7 @@
         <v>Paid Digital Ads</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15">
+    <row r="3" spans="1:10">
       <c r="A3" s="44" t="s">
         <v>721</v>
       </c>
@@ -11894,7 +11891,7 @@
         <v>Content Syndication</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15">
+    <row r="4" spans="1:10">
       <c r="A4" s="44" t="s">
         <v>724</v>
       </c>
@@ -11926,7 +11923,7 @@
         <v>Web</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15">
+    <row r="5" spans="1:10">
       <c r="A5" s="44" t="s">
         <v>726</v>
       </c>
@@ -11943,7 +11940,7 @@
         <v>Above the Line - Non Digital</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15">
+    <row r="6" spans="1:10">
       <c r="A6" s="44" t="s">
         <v>729</v>
       </c>
@@ -11966,7 +11963,7 @@
         <v>Social Posts</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15">
+    <row r="7" spans="1:10">
       <c r="A7" s="44" t="s">
         <v>730</v>
       </c>
@@ -11992,7 +11989,7 @@
         <v>Social Outbound Messages</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15">
+    <row r="8" spans="1:10">
       <c r="A8" s="44" t="s">
         <v>734</v>
       </c>
@@ -12015,7 +12012,7 @@
         <v>Virtual Events</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15">
+    <row r="9" spans="1:10">
       <c r="A9" s="44" t="s">
         <v>737</v>
       </c>
@@ -12035,7 +12032,7 @@
         <v>F2F Events</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15">
+    <row r="10" spans="1:10">
       <c r="A10" s="44" t="s">
         <v>738</v>
       </c>
@@ -12058,7 +12055,7 @@
         <v>Webinars</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15">
+    <row r="11" spans="1:10">
       <c r="A11" s="44" t="s">
         <v>739</v>
       </c>
@@ -12081,7 +12078,7 @@
         <v>Direct Mail</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15">
+    <row r="12" spans="1:10">
       <c r="A12" s="44" t="s">
         <v>740</v>
       </c>
@@ -12113,7 +12110,7 @@
         <v>Whatsapp</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15">
+    <row r="13" spans="1:10">
       <c r="A13" s="44" t="s">
         <v>741</v>
       </c>
@@ -12145,7 +12142,7 @@
         <v>RCS</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15">
+    <row r="14" spans="1:10">
       <c r="A14" s="44" t="s">
         <v>742</v>
       </c>
@@ -12179,7 +12176,7 @@
         <v>Email</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15">
+    <row r="15" spans="1:10">
       <c r="A15" s="44" t="s">
         <v>743</v>
       </c>
@@ -12211,7 +12208,7 @@
         <v>SMS</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15">
+    <row r="16" spans="1:10">
       <c r="A16" s="44" t="s">
         <v>744</v>
       </c>
@@ -12243,7 +12240,7 @@
         <v>MMS</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15">
+    <row r="17" spans="1:10">
       <c r="A17" s="44" t="s">
         <v>745</v>
       </c>
@@ -12266,7 +12263,7 @@
         <v>App Push Notification</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15">
+    <row r="18" spans="1:10">
       <c r="A18" s="44" t="s">
         <v>750</v>
       </c>
@@ -12286,7 +12283,7 @@
         <v>Sales Meetings</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15">
+    <row r="19" spans="1:10">
       <c r="A19" s="44" t="s">
         <v>752</v>
       </c>
@@ -12309,7 +12306,7 @@
         <v>Sales Calls</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15">
+    <row r="20" spans="1:10">
       <c r="A20" s="44" t="s">
         <v>753</v>
       </c>
@@ -12343,7 +12340,7 @@
         <v>Sales Email</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15">
+    <row r="21" spans="1:10">
       <c r="A21" s="45" t="s">
         <v>754</v>
       </c>
@@ -12365,7 +12362,7 @@
         <v>Inbound Calls</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15">
+    <row r="22" spans="1:10">
       <c r="A22" s="44" t="s">
         <v>746</v>
       </c>
@@ -12420,6 +12417,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D1F78A46A5B61544A3F5E5F9D558353B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd5889db134979e54dcf054cdc4727ec">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7019f60-298e-442e-b6f6-687001478962" xmlns:ns3="244a3a2d-c3b8-4eaa-9334-4c3b8cbc7cc9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdf5543a8e45e11fa247a01810ff6e7b" ns2:_="" ns3:_="">
     <xsd:import namespace="a7019f60-298e-442e-b6f6-687001478962"/>
@@ -12620,29 +12632,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221E8208-2559-4473-AFD3-FB4000FD0DD1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{981D98BA-C602-41F7-9CF6-ADC2B2B0572D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{981D98BA-C602-41F7-9CF6-ADC2B2B0572D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51BB428E-D1CA-47E8-B784-F33B49A13D8D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51BB428E-D1CA-47E8-B784-F33B49A13D8D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{221E8208-2559-4473-AFD3-FB4000FD0DD1}"/>
 </file>
</xml_diff>